<commit_message>
Database update: Database-V-28-05-2026.xlsx via Streamlit
</commit_message>
<xml_diff>
--- a/Database-V-28-05-2026.xlsx
+++ b/Database-V-28-05-2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sightlinemedia-my.sharepoint.com/personal/lconord_lydech_com/Documents/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32278572-2A49-4000-B46D-EAF66EA6F325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{32278572-2A49-4000-B46D-EAF66EA6F325}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE155A01-8333-4BD4-A710-C0B13C5070A9}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GNRL Characteristics" sheetId="1" r:id="rId1"/>
@@ -3913,7 +3913,7 @@
         <v>1400</v>
       </c>
       <c r="O27" s="8">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="P27" s="10" t="s">
         <v>40</v>

</xml_diff>